<commit_message>
adds more nzlum style build artefacts
</commit_message>
<xml_diff>
--- a/classification-systems/nzlum/build/0.3.0/nzlum_v0.3.0.xlsx
+++ b/classification-systems/nzlum/build/0.3.0/nzlum_v0.3.0.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NZLUM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NZLUM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2823,74 +2823,74 @@
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="E66:E71"/>
-    <mergeCell ref="E27:E29"/>
-    <mergeCell ref="F53:F56"/>
+    <mergeCell ref="A2:A21"/>
+    <mergeCell ref="A22:A52"/>
+    <mergeCell ref="A53:A96"/>
+    <mergeCell ref="B2:B21"/>
+    <mergeCell ref="B22:B52"/>
+    <mergeCell ref="B53:B96"/>
+    <mergeCell ref="D2:D8"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D12:D19"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D26"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D39:D43"/>
+    <mergeCell ref="D44:D48"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="D57:D59"/>
     <mergeCell ref="D60:D65"/>
-    <mergeCell ref="E12:E19"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="D66:D71"/>
     <mergeCell ref="D72:D78"/>
-    <mergeCell ref="F72:F78"/>
-    <mergeCell ref="E89:E93"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="F22:F26"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="F27:F29"/>
-    <mergeCell ref="D49:D52"/>
-    <mergeCell ref="E2:E8"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="F57:F59"/>
-    <mergeCell ref="D39:D43"/>
-    <mergeCell ref="E84:E88"/>
-    <mergeCell ref="A2:A21"/>
-    <mergeCell ref="E60:E65"/>
     <mergeCell ref="D79:D83"/>
-    <mergeCell ref="F39:F43"/>
-    <mergeCell ref="F49:F52"/>
-    <mergeCell ref="E72:E78"/>
+    <mergeCell ref="D84:D88"/>
     <mergeCell ref="D89:D93"/>
     <mergeCell ref="D94:D96"/>
+    <mergeCell ref="E2:E8"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="E12:E19"/>
+    <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E26"/>
-    <mergeCell ref="B53:B96"/>
-    <mergeCell ref="A22:A52"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="E39:E43"/>
+    <mergeCell ref="E44:E48"/>
     <mergeCell ref="E49:E52"/>
+    <mergeCell ref="E53:E56"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="E60:E65"/>
+    <mergeCell ref="E66:E71"/>
+    <mergeCell ref="E72:E78"/>
+    <mergeCell ref="E79:E83"/>
+    <mergeCell ref="E84:E88"/>
+    <mergeCell ref="E89:E93"/>
+    <mergeCell ref="E94:E96"/>
+    <mergeCell ref="F9:F11"/>
     <mergeCell ref="F12:F19"/>
-    <mergeCell ref="D44:D48"/>
-    <mergeCell ref="D66:D71"/>
-    <mergeCell ref="D22:D26"/>
-    <mergeCell ref="D84:D88"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="A53:A96"/>
-    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F22:F26"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="F30:F33"/>
     <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F43"/>
     <mergeCell ref="F44:F48"/>
+    <mergeCell ref="F49:F52"/>
+    <mergeCell ref="F53:F56"/>
+    <mergeCell ref="F57:F59"/>
+    <mergeCell ref="F60:F65"/>
     <mergeCell ref="F66:F71"/>
+    <mergeCell ref="F72:F78"/>
+    <mergeCell ref="F79:F83"/>
     <mergeCell ref="F84:F88"/>
-    <mergeCell ref="E79:E83"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D27:D29"/>
-    <mergeCell ref="E94:E96"/>
-    <mergeCell ref="E39:E43"/>
-    <mergeCell ref="B22:B52"/>
-    <mergeCell ref="F60:F65"/>
-    <mergeCell ref="E44:E48"/>
-    <mergeCell ref="D12:D19"/>
-    <mergeCell ref="D57:D59"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F79:F83"/>
-    <mergeCell ref="E37:E38"/>
     <mergeCell ref="F89:F93"/>
     <mergeCell ref="F94:F96"/>
-    <mergeCell ref="D2:D8"/>
-    <mergeCell ref="B2:B21"/>
-    <mergeCell ref="E53:E56"/>
-    <mergeCell ref="E9:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>